<commit_message>
Fill xlsx Requirements/Acceptance sheets; catch a real TR03 overclaim
58 requirements and 23 acceptance criteria filled with per-item verified
evidence (commit, test name, or a grep run this session) -- 34/8/16 and
7/10/6 Pass/Partial/Not-tested respectively.

Checking REQ-020 on its own, rather than trusting the WP-level TR03 pass
that bundled it with REQ-021, found its not-applicable-vs-class-floor
validation has zero implementation anywhere in backend/app/. Corrected TR03
to Partial and logged a new open finding in docs/DEFECT_REGISTER.md. Also
fixed two stale "not yet committed" citations now that the prior session's
work is actually on origin.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/blueprint/Build_Governance_Platform_Implementation_Tracker_v0.2_Approved.xlsx
+++ b/docs/blueprint/Build_Governance_Platform_Implementation_Tracker_v0.2_Approved.xlsx
@@ -885,10 +885,14 @@
       </c>
       <c r="I6" s="7" t="inlineStr">
         <is>
-          <t>Not tested</t>
-        </is>
-      </c>
-      <c r="J6" s="7" t="str"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J6" s="7" t="inlineStr">
+        <is>
+          <t>commit deb3969 (WP03); explicit organisation membership created at registration; test_identity.py registration tests</t>
+        </is>
+      </c>
       <c r="K6" s="7" t="str"/>
       <c r="L6" s="4">
         <f>IF(AND(I6="Pass",J6&lt;&gt;"",K6&lt;&gt;""),"Verified","Unverified")</f>
@@ -941,11 +945,19 @@
       </c>
       <c r="I7" s="7" t="inlineStr">
         <is>
-          <t>Not tested</t>
-        </is>
-      </c>
-      <c r="J7" s="7" t="str"/>
-      <c r="K7" s="7" t="str"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J7" s="7" t="inlineStr">
+        <is>
+          <t>require_mfa dependency (app/deps.py) gates approval authority; BGP-F01 fix (b1fb402) made login session-bound to a real second-factor check, not an account flag; test_hardening.py MFA-session tests</t>
+        </is>
+      </c>
+      <c r="K7" s="7" t="inlineStr">
+        <is>
+          <t>MiltonBello15 (PR#3, BGP-F01 fix -- APPROVED)</t>
+        </is>
+      </c>
       <c r="L7" s="4">
         <f>IF(AND(I7="Pass",J7&lt;&gt;"",K7&lt;&gt;""),"Verified","Unverified")</f>
         <v/>
@@ -997,11 +1009,19 @@
       </c>
       <c r="I8" s="7" t="inlineStr">
         <is>
-          <t>Not tested</t>
-        </is>
-      </c>
-      <c r="J8" s="7" t="str"/>
-      <c r="K8" s="7" t="str"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J8" s="7" t="inlineStr">
+        <is>
+          <t>Active tenant resolved from server session (app/deps.py); org-bootstrap RLS-context-ordering bug in get_active_membership fixed PR#4 (ac7f0f1)</t>
+        </is>
+      </c>
+      <c r="K8" s="7" t="inlineStr">
+        <is>
+          <t>MiltonBello15 (PR#4 -- APPROVED)</t>
+        </is>
+      </c>
       <c r="L8" s="4">
         <f>IF(AND(I8="Pass",J8&lt;&gt;"",K8&lt;&gt;""),"Verified","Unverified")</f>
         <v/>
@@ -1053,10 +1073,14 @@
       </c>
       <c r="I9" s="7" t="inlineStr">
         <is>
-          <t>Not tested</t>
-        </is>
-      </c>
-      <c r="J9" s="7" t="str"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J9" s="7" t="inlineStr">
+        <is>
+          <t>require_role()/membership checks enforced per router (backend/app/routers/*.py); RLS-backed tests across test_wp0*_tenant_isolation_rls.py</t>
+        </is>
+      </c>
       <c r="K9" s="7" t="str"/>
       <c r="L9" s="4">
         <f>IF(AND(I9="Pass",J9&lt;&gt;"",K9&lt;&gt;""),"Verified","Unverified")</f>
@@ -1109,10 +1133,14 @@
       </c>
       <c r="I10" s="7" t="inlineStr">
         <is>
-          <t>Not tested</t>
-        </is>
-      </c>
-      <c r="J10" s="7" t="str"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J10" s="7" t="inlineStr">
+        <is>
+          <t>GET /orgs/{tenant_id}/access-review (app/routers/orgs.py:232); test_access_review_lists_tenant_membership + test_access_review_requires_tenant_administrator_role</t>
+        </is>
+      </c>
       <c r="K10" s="7" t="str"/>
       <c r="L10" s="4">
         <f>IF(AND(I10="Pass",J10&lt;&gt;"",K10&lt;&gt;""),"Verified","Unverified")</f>
@@ -1165,11 +1193,19 @@
       </c>
       <c r="I11" s="7" t="inlineStr">
         <is>
-          <t>Not tested</t>
-        </is>
-      </c>
-      <c r="J11" s="7" t="str"/>
-      <c r="K11" s="7" t="str"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J11" s="7" t="inlineStr">
+        <is>
+          <t>Compensating review now created from the reviewer's own authenticated, MFA-verified session (BGP-F02 fix, b1fb402); preparer-set-from-ownership bypass closed by the follow-up fix (b8bb22a, PR#3): test_clearing_or_reassigning_ownership_cannot_defeat_separation_of_duties</t>
+        </is>
+      </c>
+      <c r="K11" s="7" t="inlineStr">
+        <is>
+          <t>MiltonBello15 (PR#3, BGP-F02 + follow-up fix -- APPROVED)</t>
+        </is>
+      </c>
       <c r="L11" s="4">
         <f>IF(AND(I11="Pass",J11&lt;&gt;"",K11&lt;&gt;""),"Verified","Unverified")</f>
         <v/>
@@ -1221,10 +1257,14 @@
       </c>
       <c r="I12" s="7" t="inlineStr">
         <is>
-          <t>Not tested</t>
-        </is>
-      </c>
-      <c r="J12" s="7" t="str"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J12" s="7" t="inlineStr">
+        <is>
+          <t>tenant_id on every owned row; RLS migrations 0002 (WP04) and 0014 (org-bootstrap fix, PR#4); adversarial cross-tenant suite passing against real Postgres</t>
+        </is>
+      </c>
       <c r="K12" s="7" t="str"/>
       <c r="L12" s="4">
         <f>IF(AND(I12="Pass",J12&lt;&gt;"",K12&lt;&gt;""),"Verified","Unverified")</f>
@@ -1277,10 +1317,14 @@
       </c>
       <c r="I13" s="7" t="inlineStr">
         <is>
-          <t>Not tested</t>
-        </is>
-      </c>
-      <c r="J13" s="7" t="str"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J13" s="7" t="inlineStr">
+        <is>
+          <t>SET LOCAL app.tenant_id reset per request (app/deps.py); pooled-connection tenant-reset test in test_tenant_isolation_rls.py</t>
+        </is>
+      </c>
       <c r="K13" s="7" t="str"/>
       <c r="L13" s="4">
         <f>IF(AND(I13="Pass",J13&lt;&gt;"",K13&lt;&gt;""),"Verified","Unverified")</f>
@@ -1333,10 +1377,14 @@
       </c>
       <c r="I14" s="7" t="inlineStr">
         <is>
-          <t>Not tested</t>
-        </is>
-      </c>
-      <c r="J14" s="7" t="str"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J14" s="7" t="inlineStr">
+        <is>
+          <t>Adversarial cross-tenant suite is a real, currently-green, CI-blocking check -- confirmed live via gh run view on run 35670396664, 2026-09-24</t>
+        </is>
+      </c>
       <c r="K14" s="7" t="str"/>
       <c r="L14" s="4">
         <f>IF(AND(I14="Pass",J14&lt;&gt;"",K14&lt;&gt;""),"Verified","Unverified")</f>
@@ -1389,10 +1437,14 @@
       </c>
       <c r="I15" s="7" t="inlineStr">
         <is>
-          <t>Not tested</t>
-        </is>
-      </c>
-      <c r="J15" s="7" t="str"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J15" s="7" t="inlineStr">
+        <is>
+          <t>Template versioning in app/rule_engine.py + templates router; create/publish tested</t>
+        </is>
+      </c>
       <c r="K15" s="7" t="str"/>
       <c r="L15" s="4">
         <f>IF(AND(I15="Pass",J15&lt;&gt;"",K15&lt;&gt;""),"Verified","Unverified")</f>
@@ -1445,10 +1497,14 @@
       </c>
       <c r="I16" s="7" t="inlineStr">
         <is>
-          <t>Not tested</t>
-        </is>
-      </c>
-      <c r="J16" s="7" t="str"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J16" s="7" t="inlineStr">
+        <is>
+          <t>Publish-time immutability enforced; changing a published template creates a new version, tested</t>
+        </is>
+      </c>
       <c r="K16" s="7" t="str"/>
       <c r="L16" s="4">
         <f>IF(AND(I16="Pass",J16&lt;&gt;"",K16&lt;&gt;""),"Verified","Unverified")</f>
@@ -1501,10 +1557,14 @@
       </c>
       <c r="I17" s="7" t="inlineStr">
         <is>
-          <t>Not tested</t>
-        </is>
-      </c>
-      <c r="J17" s="7" t="str"/>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="J17" s="7" t="inlineStr">
+        <is>
+          <t>fork_template/import_template (app/routers/templates.py:171,205) and create-blank are real, tested backend endpoints, but the guided-authoring UI (UI08) has no frontend page yet -- open as IPA02 in BGP_Implementation_Plan_Alignment_Findings_v1.0.docx</t>
+        </is>
+      </c>
       <c r="K17" s="7" t="str"/>
       <c r="L17" s="4">
         <f>IF(AND(I17="Pass",J17&lt;&gt;"",K17&lt;&gt;""),"Verified","Unverified")</f>
@@ -1557,10 +1617,14 @@
       </c>
       <c r="I18" s="7" t="inlineStr">
         <is>
-          <t>Not tested</t>
-        </is>
-      </c>
-      <c r="J18" s="7" t="str"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J18" s="7" t="inlineStr">
+        <is>
+          <t>app/rule_engine.py restricted to eq/in/all/any vocabulary only, no eval/exec, depth limit 5</t>
+        </is>
+      </c>
       <c r="K18" s="7" t="str"/>
       <c r="L18" s="4">
         <f>IF(AND(I18="Pass",J18&lt;&gt;"",K18&lt;&gt;""),"Verified","Unverified")</f>
@@ -1613,10 +1677,14 @@
       </c>
       <c r="I19" s="7" t="inlineStr">
         <is>
-          <t>Not tested</t>
-        </is>
-      </c>
-      <c r="J19" s="7" t="str"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J19" s="7" t="inlineStr">
+        <is>
+          <t>No real KenAddme content used; 3 neutral fictional framework fixtures (fixtures/synthetic/frameworks/) per DEC03's still-open licensing gate</t>
+        </is>
+      </c>
       <c r="K19" s="7" t="str"/>
       <c r="L19" s="4">
         <f>IF(AND(I19="Pass",J19&lt;&gt;"",K19&lt;&gt;""),"Verified","Unverified")</f>
@@ -1669,10 +1737,14 @@
       </c>
       <c r="I20" s="7" t="inlineStr">
         <is>
-          <t>Not tested</t>
-        </is>
-      </c>
-      <c r="J20" s="7" t="str"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J20" s="7" t="inlineStr">
+        <is>
+          <t>Atomic project seeding proven by test_seeding_failure_leaves_no_project_row (monkeypatches mid-seed failure, asserts zero rows persist)</t>
+        </is>
+      </c>
       <c r="K20" s="7" t="str"/>
       <c r="L20" s="4">
         <f>IF(AND(I20="Pass",J20&lt;&gt;"",K20&lt;&gt;""),"Verified","Unverified")</f>
@@ -1725,10 +1797,14 @@
       </c>
       <c r="I21" s="7" t="inlineStr">
         <is>
-          <t>Not tested</t>
-        </is>
-      </c>
-      <c r="J21" s="7" t="str"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J21" s="7" t="inlineStr">
+        <is>
+          <t>gate_occurrences table represents every routine/triggered review as its own row (WP06)</t>
+        </is>
+      </c>
       <c r="K21" s="7" t="str"/>
       <c r="L21" s="4">
         <f>IF(AND(I21="Pass",J21&lt;&gt;"",K21&lt;&gt;""),"Verified","Unverified")</f>
@@ -1781,10 +1857,14 @@
       </c>
       <c r="I22" s="7" t="inlineStr">
         <is>
-          <t>Not tested</t>
-        </is>
-      </c>
-      <c r="J22" s="7" t="str"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J22" s="7" t="inlineStr">
+        <is>
+          <t>evidence_items track status/owner/due date/completion date/reference (WP06)</t>
+        </is>
+      </c>
       <c r="K22" s="7" t="str"/>
       <c r="L22" s="4">
         <f>IF(AND(I22="Pass",J22&lt;&gt;"",K22&lt;&gt;""),"Verified","Unverified")</f>
@@ -1837,10 +1917,14 @@
       </c>
       <c r="I23" s="7" t="inlineStr">
         <is>
-          <t>Not tested</t>
-        </is>
-      </c>
-      <c r="J23" s="7" t="str"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J23" s="7" t="inlineStr">
+        <is>
+          <t>status=Complete+required+no-reference rejected at the API boundary, enforced and tested</t>
+        </is>
+      </c>
       <c r="K23" s="7" t="str"/>
       <c r="L23" s="4">
         <f>IF(AND(I23="Pass",J23&lt;&gt;"",K23&lt;&gt;""),"Verified","Unverified")</f>
@@ -1893,11 +1977,19 @@
       </c>
       <c r="I24" s="7" t="inlineStr">
         <is>
-          <t>Not tested</t>
-        </is>
-      </c>
-      <c r="J24" s="7" t="str"/>
-      <c r="K24" s="7" t="str"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J24" s="7" t="inlineStr">
+        <is>
+          <t>source_version/source_hash are explicit disclosed fields, never inferred; preserved through export/import re-hops per BGP-F04 fix (b1fb402) and follow-up fix (b8bb22a)</t>
+        </is>
+      </c>
+      <c r="K24" s="7" t="inlineStr">
+        <is>
+          <t>MiltonBello15 (PR#3, BGP-F04 follow-up fix -- APPROVED)</t>
+        </is>
+      </c>
       <c r="L24" s="4">
         <f>IF(AND(I24="Pass",J24&lt;&gt;"",K24&lt;&gt;""),"Verified","Unverified")</f>
         <v/>
@@ -1952,7 +2044,11 @@
           <t>Not tested</t>
         </is>
       </c>
-      <c r="J25" s="7" t="str"/>
+      <c r="J25" s="7" t="inlineStr">
+        <is>
+          <t>Grep-confirmed 2026-09-24: zero occurrences of 'Not applicable' classification-vs-class-floor validation logic anywhere in backend/app/. This is genuinely unbuilt, not just unverified -- a real gap this per-requirement pass caught that the WP-level Remediation-sheet pass (TR03) had missed.</t>
+        </is>
+      </c>
       <c r="K25" s="7" t="str"/>
       <c r="L25" s="4">
         <f>IF(AND(I25="Pass",J25&lt;&gt;"",K25&lt;&gt;""),"Verified","Unverified")</f>
@@ -2005,10 +2101,14 @@
       </c>
       <c r="I26" s="7" t="inlineStr">
         <is>
-          <t>Not tested</t>
-        </is>
-      </c>
-      <c r="J26" s="7" t="str"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J26" s="7" t="inlineStr">
+        <is>
+          <t>Exception create/revoke endpoints re-check authority/scope/expiry live on every call (app/routers/decisions.py), never trusted from a stored status field alone</t>
+        </is>
+      </c>
       <c r="K26" s="7" t="str"/>
       <c r="L26" s="4">
         <f>IF(AND(I26="Pass",J26&lt;&gt;"",K26&lt;&gt;""),"Verified","Unverified")</f>
@@ -2061,10 +2161,14 @@
       </c>
       <c r="I27" s="7" t="inlineStr">
         <is>
-          <t>Not tested</t>
-        </is>
-      </c>
-      <c r="J27" s="7" t="str"/>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="J27" s="7" t="inlineStr">
+        <is>
+          <t>Conditions are recorded and required before a conditional approval, but REQ-022's own 'activity limits' on what a conditionally-approved project can then do are not enforced -- an open gap named in the WP07 build notes since 2026-09-16 (TR04)</t>
+        </is>
+      </c>
       <c r="K27" s="7" t="str"/>
       <c r="L27" s="4">
         <f>IF(AND(I27="Pass",J27&lt;&gt;"",K27&lt;&gt;""),"Verified","Unverified")</f>
@@ -2117,10 +2221,14 @@
       </c>
       <c r="I28" s="7" t="inlineStr">
         <is>
-          <t>Not tested</t>
-        </is>
-      </c>
-      <c r="J28" s="7" t="str"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J28" s="7" t="inlineStr">
+        <is>
+          <t>decision_records is a SELECT+INSERT-only DB-role grant (not just a route-level check); test_wp07_tenant_isolation_rls.py proves UPDATE/DELETE both raise permission denied</t>
+        </is>
+      </c>
       <c r="K28" s="7" t="str"/>
       <c r="L28" s="4">
         <f>IF(AND(I28="Pass",J28&lt;&gt;"",K28&lt;&gt;""),"Verified","Unverified")</f>
@@ -2173,11 +2281,19 @@
       </c>
       <c r="I29" s="7" t="inlineStr">
         <is>
-          <t>Not tested</t>
-        </is>
-      </c>
-      <c r="J29" s="7" t="str"/>
-      <c r="K29" s="7" t="str"/>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="J29" s="7" t="inlineStr">
+        <is>
+          <t>Evidence-row and project-membership-row locking added (BGP-F03 fix b1fb402 + follow-up b8bb22a, PR#3/#4). Still open per BGP-IPA-001/IPA04, confirmed against source: exception validity, tenant membership and compensating-reviewer authority are read without equivalent coordinated (locked) protection on the decision-commit path.</t>
+        </is>
+      </c>
+      <c r="K29" s="7" t="inlineStr">
+        <is>
+          <t>MiltonBello15 (PR#3/#4, concurrency fixes -- APPROVED; gap remains beyond what those PRs fixed)</t>
+        </is>
+      </c>
       <c r="L29" s="4">
         <f>IF(AND(I29="Pass",J29&lt;&gt;"",K29&lt;&gt;""),"Verified","Unverified")</f>
         <v/>
@@ -2229,10 +2345,14 @@
       </c>
       <c r="I30" s="7" t="inlineStr">
         <is>
-          <t>Not tested</t>
-        </is>
-      </c>
-      <c r="J30" s="7" t="str"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J30" s="7" t="inlineStr">
+        <is>
+          <t>Superseding endpoint never mutates the original row; a reason is mandatory; original-decision reference preserved</t>
+        </is>
+      </c>
       <c r="K30" s="7" t="str"/>
       <c r="L30" s="4">
         <f>IF(AND(I30="Pass",J30&lt;&gt;"",K30&lt;&gt;""),"Verified","Unverified")</f>
@@ -2285,10 +2405,14 @@
       </c>
       <c r="I31" s="7" t="inlineStr">
         <is>
-          <t>Not tested</t>
-        </is>
-      </c>
-      <c r="J31" s="7" t="str"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J31" s="7" t="inlineStr">
+        <is>
+          <t>integrity_checkpoints hash chain (WP08); the bgp_owner Postgres-superuser RLS-bypass bug was found and fixed the same session it was discovered</t>
+        </is>
+      </c>
       <c r="K31" s="7" t="str"/>
       <c r="L31" s="4">
         <f>IF(AND(I31="Pass",J31&lt;&gt;"",K31&lt;&gt;""),"Verified","Unverified")</f>
@@ -2341,10 +2465,14 @@
       </c>
       <c r="I32" s="7" t="inlineStr">
         <is>
-          <t>Not tested</t>
-        </is>
-      </c>
-      <c r="J32" s="7" t="str"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J32" s="7" t="inlineStr">
+        <is>
+          <t>An open integrity incident blocks new decisions project-wide, HTTP 423 (WP08)</t>
+        </is>
+      </c>
       <c r="K32" s="7" t="str"/>
       <c r="L32" s="4">
         <f>IF(AND(I32="Pass",J32&lt;&gt;"",K32&lt;&gt;""),"Verified","Unverified")</f>
@@ -2400,7 +2528,11 @@
           <t>Not tested</t>
         </is>
       </c>
-      <c r="J33" s="7" t="str"/>
+      <c r="J33" s="7" t="inlineStr">
+        <is>
+          <t>Only a local-atomicity fault test exists (crash-at-commit leaves zero partial rows). The review's own text is explicit this is 'not a node/zone/region durability proof', and DEC05 (the actual approved failure envelope) remains unresolved -- so REQ-028's specific claim (zero loss within the APPROVED envelope) cannot be marked Pass without an envelope to test against.</t>
+        </is>
+      </c>
       <c r="K33" s="7" t="str"/>
       <c r="L33" s="4">
         <f>IF(AND(I33="Pass",J33&lt;&gt;"",K33&lt;&gt;""),"Verified","Unverified")</f>
@@ -2453,10 +2585,14 @@
       </c>
       <c r="I34" s="7" t="inlineStr">
         <is>
-          <t>Not tested</t>
-        </is>
-      </c>
-      <c r="J34" s="7" t="str"/>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="J34" s="7" t="inlineStr">
+        <is>
+          <t>backend/scripts/restore_drill.py actually run against live bgp_dev with real numbers (backup 1.18s / restore 4.14s / 16-table reconciliation, 2026-09-17). Explicitly scoped as a local-prototype-only result, not proof of the approved envelope's RPO/RTO since DEC05 is still open.</t>
+        </is>
+      </c>
       <c r="K34" s="7" t="str"/>
       <c r="L34" s="4">
         <f>IF(AND(I34="Pass",J34&lt;&gt;"",K34&lt;&gt;""),"Verified","Unverified")</f>
@@ -2509,11 +2645,19 @@
       </c>
       <c r="I35" s="7" t="inlineStr">
         <is>
-          <t>Not tested</t>
-        </is>
-      </c>
-      <c r="J35" s="7" t="str"/>
-      <c r="K35" s="7" t="str"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J35" s="7" t="inlineStr">
+        <is>
+          <t>Full evidence-revision history, source_id provenance across export/import hops, decision-manifest/compensating-review export -- fixed via BGP-F04 (b1fb402) and follow-up (b8bb22a, PR#3): test_unmatched_revision_author_and_timestamp_survive_reexport</t>
+        </is>
+      </c>
+      <c r="K35" s="7" t="inlineStr">
+        <is>
+          <t>MiltonBello15 (PR#3 -- APPROVED)</t>
+        </is>
+      </c>
       <c r="L35" s="4">
         <f>IF(AND(I35="Pass",J35&lt;&gt;"",K35&lt;&gt;""),"Verified","Unverified")</f>
         <v/>
@@ -2565,10 +2709,14 @@
       </c>
       <c r="I36" s="7" t="inlineStr">
         <is>
-          <t>Not tested</t>
-        </is>
-      </c>
-      <c r="J36" s="7" t="str"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J36" s="7" t="inlineStr">
+        <is>
+          <t>Any active project member can export their own data -- explicitly documented in app/routers/exports.py's own REQ-031 comment (line 443) and exercised by test_export_import.py</t>
+        </is>
+      </c>
       <c r="K36" s="7" t="str"/>
       <c r="L36" s="4">
         <f>IF(AND(I36="Pass",J36&lt;&gt;"",K36&lt;&gt;""),"Verified","Unverified")</f>
@@ -2621,10 +2769,14 @@
       </c>
       <c r="I37" s="7" t="inlineStr">
         <is>
-          <t>Not tested</t>
-        </is>
-      </c>
-      <c r="J37" s="7" t="str"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J37" s="7" t="inlineStr">
+        <is>
+          <t>GET /my-work wraps each item with project_name/reason/direct_action (WP10); my_work.html real page (WP11-heading frontend increment)</t>
+        </is>
+      </c>
       <c r="K37" s="7" t="str"/>
       <c r="L37" s="4">
         <f>IF(AND(I37="Pass",J37&lt;&gt;"",K37&lt;&gt;""),"Verified","Unverified")</f>
@@ -2677,10 +2829,14 @@
       </c>
       <c r="I38" s="7" t="inlineStr">
         <is>
-          <t>Not tested</t>
-        </is>
-      </c>
-      <c r="J38" s="7" t="str"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J38" s="7" t="inlineStr">
+        <is>
+          <t>Guided forms with plain 'Back to My work' links present in evidence_form.html, project_new.html, decide.html -- grep-confirmed 2026-09-24</t>
+        </is>
+      </c>
       <c r="K38" s="7" t="str"/>
       <c r="L38" s="4">
         <f>IF(AND(I38="Pass",J38&lt;&gt;"",K38&lt;&gt;""),"Verified","Unverified")</f>
@@ -2733,10 +2889,14 @@
       </c>
       <c r="I39" s="7" t="inlineStr">
         <is>
-          <t>Not tested</t>
-        </is>
-      </c>
-      <c r="J39" s="7" t="str"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J39" s="7" t="inlineStr">
+        <is>
+          <t>drafts table, save/resume with Saving/Saved/Not saved states (WP10), tested</t>
+        </is>
+      </c>
       <c r="K39" s="7" t="str"/>
       <c r="L39" s="4">
         <f>IF(AND(I39="Pass",J39&lt;&gt;"",K39&lt;&gt;""),"Verified","Unverified")</f>
@@ -2792,7 +2952,11 @@
           <t>Not tested</t>
         </is>
       </c>
-      <c r="J40" s="7" t="str"/>
+      <c r="J40" s="7" t="inlineStr">
+        <is>
+          <t>decide_submit (app/webapp/router.py:578) generates a fresh uuid.uuid4() idempotency key on every submission -- grep-reconfirmed 2026-09-24. IPA03's finding stands: the browser-facing pending/confirmed-approval recovery this requirement asks for does not exist, even though the underlying JSON API's own idempotency handling (WP07) is correct.</t>
+        </is>
+      </c>
       <c r="K40" s="7" t="str"/>
       <c r="L40" s="4">
         <f>IF(AND(I40="Pass",J40&lt;&gt;"",K40&lt;&gt;""),"Verified","Unverified")</f>
@@ -2845,10 +3009,14 @@
       </c>
       <c r="I41" s="7" t="inlineStr">
         <is>
-          <t>Not tested</t>
-        </is>
-      </c>
-      <c r="J41" s="7" t="str"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J41" s="7" t="inlineStr">
+        <is>
+          <t>blocker_explanations: plain-language reason + corrective-action API call per blocker (WP10 preview endpoint)</t>
+        </is>
+      </c>
       <c r="K41" s="7" t="str"/>
       <c r="L41" s="4">
         <f>IF(AND(I41="Pass",J41&lt;&gt;"",K41&lt;&gt;""),"Verified","Unverified")</f>
@@ -2901,10 +3069,14 @@
       </c>
       <c r="I42" s="7" t="inlineStr">
         <is>
-          <t>Not tested</t>
-        </is>
-      </c>
-      <c r="J42" s="7" t="str"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J42" s="7" t="inlineStr">
+        <is>
+          <t>Decision preview shows evidence, conditions and permitted_outcomes (every outcome current readiness would allow), WP10</t>
+        </is>
+      </c>
       <c r="K42" s="7" t="str"/>
       <c r="L42" s="4">
         <f>IF(AND(I42="Pass",J42&lt;&gt;"",K42&lt;&gt;""),"Verified","Unverified")</f>
@@ -2957,10 +3129,14 @@
       </c>
       <c r="I43" s="7" t="inlineStr">
         <is>
-          <t>Not tested</t>
-        </is>
-      </c>
-      <c r="J43" s="7" t="str"/>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="J43" s="7" t="inlineStr">
+        <is>
+          <t>Accessible MFA setup/verify and recovery-code flow are real and tested (mfa_enroll.html, mfa_login_verify.html). No dedicated 'invitation landing' HTML page exists though -- accept_invitation (app/routers/orgs.py:130) is API-only, grep-confirmed no matching template in backend/app/templates/.</t>
+        </is>
+      </c>
       <c r="K43" s="7" t="str"/>
       <c r="L43" s="4">
         <f>IF(AND(I43="Pass",J43&lt;&gt;"",K43&lt;&gt;""),"Verified","Unverified")</f>
@@ -3016,7 +3192,11 @@
           <t>Not tested</t>
         </is>
       </c>
-      <c r="J44" s="7" t="str"/>
+      <c r="J44" s="7" t="inlineStr">
+        <is>
+          <t>No timezone-specific handling found in any template (grep-confirmed 2026-09-24); translation structure not verified</t>
+        </is>
+      </c>
       <c r="K44" s="7" t="str"/>
       <c r="L44" s="4">
         <f>IF(AND(I44="Pass",J44&lt;&gt;"",K44&lt;&gt;""),"Verified","Unverified")</f>
@@ -3072,7 +3252,11 @@
           <t>Not tested</t>
         </is>
       </c>
-      <c r="J45" s="7" t="str"/>
+      <c r="J45" s="7" t="inlineStr">
+        <is>
+          <t>No WCAG 2.2 AA audit has been performed. Blueprint's real WP11 ('Usability and accessibility') has not started -- see docs/wp_identifier_mapping.md.</t>
+        </is>
+      </c>
       <c r="K45" s="7" t="str"/>
       <c r="L45" s="4">
         <f>IF(AND(I45="Pass",J45&lt;&gt;"",K45&lt;&gt;""),"Verified","Unverified")</f>
@@ -3128,7 +3312,11 @@
           <t>Not tested</t>
         </is>
       </c>
-      <c r="J46" s="7" t="str"/>
+      <c r="J46" s="7" t="inlineStr">
+        <is>
+          <t>No participant onboarding-time testing has been performed</t>
+        </is>
+      </c>
       <c r="K46" s="7" t="str"/>
       <c r="L46" s="4">
         <f>IF(AND(I46="Pass",J46&lt;&gt;"",K46&lt;&gt;""),"Verified","Unverified")</f>
@@ -3184,7 +3372,11 @@
           <t>Not tested</t>
         </is>
       </c>
-      <c r="J47" s="7" t="str"/>
+      <c r="J47" s="7" t="inlineStr">
+        <is>
+          <t>No critical-approval-misunderstanding testing or blocking mechanism has been built or verified</t>
+        </is>
+      </c>
       <c r="K47" s="7" t="str"/>
       <c r="L47" s="4">
         <f>IF(AND(I47="Pass",J47&lt;&gt;"",K47&lt;&gt;""),"Verified","Unverified")</f>
@@ -3240,7 +3432,11 @@
           <t>Not tested</t>
         </is>
       </c>
-      <c r="J48" s="7" t="str"/>
+      <c r="J48" s="7" t="inlineStr">
+        <is>
+          <t>REQ-043's numeric performance budget stays DEC08-gated; no real-traffic availability baseline exists for this local prototype</t>
+        </is>
+      </c>
       <c r="K48" s="7" t="str"/>
       <c r="L48" s="4">
         <f>IF(AND(I48="Pass",J48&lt;&gt;"",K48&lt;&gt;""),"Verified","Unverified")</f>
@@ -3296,7 +3492,11 @@
           <t>Not tested</t>
         </is>
       </c>
-      <c r="J49" s="7" t="str"/>
+      <c r="J49" s="7" t="inlineStr">
+        <is>
+          <t>docs/wp02/threat_model_and_privacy_assessment.md covers all 6 required categories but is Submitted for review, not independently reviewed by Milton yet</t>
+        </is>
+      </c>
       <c r="K49" s="7" t="str"/>
       <c r="L49" s="4">
         <f>IF(AND(I49="Pass",J49&lt;&gt;"",K49&lt;&gt;""),"Verified","Unverified")</f>
@@ -3349,10 +3549,14 @@
       </c>
       <c r="I50" s="7" t="inlineStr">
         <is>
-          <t>Not tested</t>
-        </is>
-      </c>
-      <c r="J50" s="7" t="str"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J50" s="7" t="inlineStr">
+        <is>
+          <t>Session-signing key moved to settings.session_secret_key (env-overridable); MFA secret Fernet-encrypted at rest with a separately-held key (WP12)</t>
+        </is>
+      </c>
       <c r="K50" s="7" t="str"/>
       <c r="L50" s="4">
         <f>IF(AND(I50="Pass",J50&lt;&gt;"",K50&lt;&gt;""),"Verified","Unverified")</f>
@@ -3405,10 +3609,14 @@
       </c>
       <c r="I51" s="7" t="inlineStr">
         <is>
-          <t>Not tested</t>
-        </is>
-      </c>
-      <c r="J51" s="7" t="str"/>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="J51" s="7" t="inlineStr">
+        <is>
+          <t>pip-audit wired into CI; 14 real known vulnerabilities were found and fixed the same session they were introduced (WP12, 2026-09-17). No ongoing 7-calendar-day remediation SLA/tracking process exists for future findings.</t>
+        </is>
+      </c>
       <c r="K51" s="7" t="str"/>
       <c r="L51" s="4">
         <f>IF(AND(I51="Pass",J51&lt;&gt;"",K51&lt;&gt;""),"Verified","Unverified")</f>
@@ -3461,10 +3669,14 @@
       </c>
       <c r="I52" s="7" t="inlineStr">
         <is>
-          <t>Not tested</t>
-        </is>
-      </c>
-      <c r="J52" s="7" t="str"/>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="J52" s="7" t="inlineStr">
+        <is>
+          <t>Access-review endpoint and security_log_events table exist (the mechanism, WP12); no quarterly review has actually been run yet (the cadence)</t>
+        </is>
+      </c>
       <c r="K52" s="7" t="str"/>
       <c r="L52" s="4">
         <f>IF(AND(I52="Pass",J52&lt;&gt;"",K52&lt;&gt;""),"Verified","Unverified")</f>
@@ -3520,7 +3732,11 @@
           <t>Not tested</t>
         </is>
       </c>
-      <c r="J53" s="7" t="str"/>
+      <c r="J53" s="7" t="inlineStr">
+        <is>
+          <t>docs/wp02/data_retention_policy.md drafted with explicitly-marked unconfirmed default floors, not an approved/confirmed policy</t>
+        </is>
+      </c>
       <c r="K53" s="7" t="str"/>
       <c r="L53" s="4">
         <f>IF(AND(I53="Pass",J53&lt;&gt;"",K53&lt;&gt;""),"Verified","Unverified")</f>
@@ -3573,11 +3789,19 @@
       </c>
       <c r="I54" s="7" t="inlineStr">
         <is>
-          <t>Not tested</t>
-        </is>
-      </c>
-      <c r="J54" s="7" t="str"/>
-      <c r="K54" s="7" t="str"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J54" s="7" t="inlineStr">
+        <is>
+          <t>Source control, 16 migrations, reproducible CI checks, and now real code review: BGP-HR-001 register, PRs 3-7, MiltonBello15/kenAddme APPROVED reviews independently verified via gh pr view</t>
+        </is>
+      </c>
+      <c r="K54" s="7" t="inlineStr">
+        <is>
+          <t>MiltonBello15 and kenAddme (BGP-HR-001, PRs 3-7 -- APPROVED)</t>
+        </is>
+      </c>
       <c r="L54" s="4">
         <f>IF(AND(I54="Pass",J54&lt;&gt;"",K54&lt;&gt;""),"Verified","Unverified")</f>
         <v/>
@@ -3632,7 +3856,11 @@
           <t>Not tested</t>
         </is>
       </c>
-      <c r="J55" s="7" t="str"/>
+      <c r="J55" s="7" t="inlineStr">
+        <is>
+          <t>No independent penetration test has been performed. Blueprint's real WP13 ('Independent acceptance and release') has not started -- see docs/wp_identifier_mapping.md.</t>
+        </is>
+      </c>
       <c r="K55" s="7" t="str"/>
       <c r="L55" s="4">
         <f>IF(AND(I55="Pass",J55&lt;&gt;"",K55&lt;&gt;""),"Verified","Unverified")</f>
@@ -3685,10 +3913,14 @@
       </c>
       <c r="I56" s="7" t="inlineStr">
         <is>
-          <t>Not tested</t>
-        </is>
-      </c>
-      <c r="J56" s="7" t="str"/>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="J56" s="7" t="inlineStr">
+        <is>
+          <t>This tracker (this xlsx + TRACKER.md + the pm-sdlc-tracker MySQL database) is the requirement-to-task-to-test evidence structure and now genuinely reflects current status. Named responsibilities partial (DEC01 done; most other DECs still open). No formal recurring Class A review cadence established yet.</t>
+        </is>
+      </c>
       <c r="K56" s="7" t="str"/>
       <c r="L56" s="4">
         <f>IF(AND(I56="Pass",J56&lt;&gt;"",K56&lt;&gt;""),"Verified","Unverified")</f>
@@ -3741,10 +3973,14 @@
       </c>
       <c r="I57" s="7" t="inlineStr">
         <is>
-          <t>Not tested</t>
-        </is>
-      </c>
-      <c r="J57" s="7" t="str"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J57" s="7" t="inlineStr">
+        <is>
+          <t>fixtures/synthetic/ used throughout; no real production data or external commitments made</t>
+        </is>
+      </c>
       <c r="K57" s="7" t="str"/>
       <c r="L57" s="4">
         <f>IF(AND(I57="Pass",J57&lt;&gt;"",K57&lt;&gt;""),"Verified","Unverified")</f>
@@ -3797,10 +4033,14 @@
       </c>
       <c r="I58" s="7" t="inlineStr">
         <is>
-          <t>Not tested</t>
-        </is>
-      </c>
-      <c r="J58" s="7" t="str"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J58" s="7" t="inlineStr">
+        <is>
+          <t>evidence_attachments table, real Cloudmersive scanning (EICAR-detected), undownloadable-until-clean gate -- delivered under TRACKER.md's 'WP15' heading; see docs/wp_identifier_mapping.md</t>
+        </is>
+      </c>
       <c r="K58" s="7" t="str"/>
       <c r="L58" s="4">
         <f>IF(AND(I58="Pass",J58&lt;&gt;"",K58&lt;&gt;""),"Verified","Unverified")</f>
@@ -3856,7 +4096,11 @@
           <t>Not tested</t>
         </is>
       </c>
-      <c r="J59" s="7" t="str"/>
+      <c r="J59" s="7" t="inlineStr">
+        <is>
+          <t>Reminders feature not built</t>
+        </is>
+      </c>
       <c r="K59" s="7" t="str"/>
       <c r="L59" s="4">
         <f>IF(AND(I59="Pass",J59&lt;&gt;"",K59&lt;&gt;""),"Verified","Unverified")</f>
@@ -3912,7 +4156,11 @@
           <t>Not tested</t>
         </is>
       </c>
-      <c r="J60" s="7" t="str"/>
+      <c r="J60" s="7" t="inlineStr">
+        <is>
+          <t>Practice-mode feature not built</t>
+        </is>
+      </c>
       <c r="K60" s="7" t="str"/>
       <c r="L60" s="4">
         <f>IF(AND(I60="Pass",J60&lt;&gt;"",K60&lt;&gt;""),"Verified","Unverified")</f>
@@ -3968,7 +4216,11 @@
           <t>Not tested</t>
         </is>
       </c>
-      <c r="J61" s="7" t="str"/>
+      <c r="J61" s="7" t="inlineStr">
+        <is>
+          <t>Billing feature not built; DEC10 (payment/tier/grace policy) still open</t>
+        </is>
+      </c>
       <c r="K61" s="7" t="str"/>
       <c r="L61" s="4">
         <f>IF(AND(I61="Pass",J61&lt;&gt;"",K61&lt;&gt;""),"Verified","Unverified")</f>
@@ -4024,7 +4276,11 @@
           <t>Not tested</t>
         </is>
       </c>
-      <c r="J62" s="7" t="str"/>
+      <c r="J62" s="7" t="inlineStr">
+        <is>
+          <t>docs/wp02/assurance_plan.md deliberately does not invent a budget or schedule; no Sponsor named to approve funding</t>
+        </is>
+      </c>
       <c r="K62" s="7" t="str"/>
       <c r="L62" s="4">
         <f>IF(AND(I62="Pass",J62&lt;&gt;"",K62&lt;&gt;""),"Verified","Unverified")</f>
@@ -4080,7 +4336,11 @@
           <t>Not tested</t>
         </is>
       </c>
-      <c r="J63" s="7" t="str"/>
+      <c r="J63" s="7" t="inlineStr">
+        <is>
+          <t>No release authorisation, migration/rollback rehearsal, runbook or monitoring handover exists. Blueprint's real WP13 has not started -- see docs/wp_identifier_mapping.md.</t>
+        </is>
+      </c>
       <c r="K63" s="7" t="str"/>
       <c r="L63" s="4">
         <f>IF(AND(I63="Pass",J63&lt;&gt;"",K63&lt;&gt;""),"Verified","Unverified")</f>
@@ -4195,7 +4455,11 @@
           <t>Not tested</t>
         </is>
       </c>
-      <c r="E6" s="7" t="str"/>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>REQ-001/014/015 pass, but REQ-041's 20-minute unaided onboarding has never been tested with a real participant</t>
+        </is>
+      </c>
       <c r="F6" s="7" t="str"/>
       <c r="G6" s="4">
         <f>IF(AND(D6="Pass",E6&lt;&gt;"",F6&lt;&gt;""),"Verified","Unverified")</f>
@@ -4221,10 +4485,14 @@
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>Not tested</t>
-        </is>
-      </c>
-      <c r="E7" s="7" t="str"/>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>Cross-tenant isolation suite passes with zero findings against real Postgres (REQ-001/003/007/008/009/053 all Pass); REQ-050 independent penetration testing has not been performed</t>
+        </is>
+      </c>
       <c r="F7" s="7" t="str"/>
       <c r="G7" s="4">
         <f>IF(AND(D7="Pass",E7&lt;&gt;"",F7&lt;&gt;""),"Verified","Unverified")</f>
@@ -4250,10 +4518,14 @@
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>Not tested</t>
-        </is>
-      </c>
-      <c r="E8" s="7" t="str"/>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>Outstanding-mandatory-evidence blocking works (REQ-022, activity-limits gap aside); REQ-020's not-applicable-vs-class-floor validation is not built at all</t>
+        </is>
+      </c>
       <c r="F8" s="7" t="str"/>
       <c r="G8" s="4">
         <f>IF(AND(D8="Pass",E8&lt;&gt;"",F8&lt;&gt;""),"Verified","Unverified")</f>
@@ -4279,10 +4551,14 @@
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>Not tested</t>
-        </is>
-      </c>
-      <c r="E9" s="7" t="str"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>REQ-019/023/025/026/027 all Pass -- decision edit/delete is refused at the DB-role level, provenance preserved, integrity failures block acknowledgement</t>
+        </is>
+      </c>
       <c r="F9" s="7" t="str"/>
       <c r="G9" s="4">
         <f>IF(AND(D9="Pass",E9&lt;&gt;"",F9&lt;&gt;""),"Verified","Unverified")</f>
@@ -4308,10 +4584,14 @@
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>Not tested</t>
-        </is>
-      </c>
-      <c r="E10" s="7" t="str"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="inlineStr">
+        <is>
+          <t>REQ-030/031/053 all Pass -- lossless export/import with provenance, self-service export, and scanned attachments all real and tested</t>
+        </is>
+      </c>
       <c r="F10" s="7" t="str"/>
       <c r="G10" s="4">
         <f>IF(AND(D10="Pass",E10&lt;&gt;"",F10&lt;&gt;""),"Verified","Unverified")</f>
@@ -4340,7 +4620,11 @@
           <t>Not tested</t>
         </is>
       </c>
-      <c r="E11" s="7" t="str"/>
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>Neither REQ-040 (WCAG 2.2 AA audit) nor REQ-050 (penetration test) has been performed</t>
+        </is>
+      </c>
       <c r="F11" s="7" t="str"/>
       <c r="G11" s="4">
         <f>IF(AND(D11="Pass",E11&lt;&gt;"",F11&lt;&gt;""),"Verified","Unverified")</f>
@@ -4369,7 +4653,11 @@
           <t>Not tested</t>
         </is>
       </c>
-      <c r="E12" s="7" t="str"/>
+      <c r="E12" s="7" t="inlineStr">
+        <is>
+          <t>REQ-028's zero-loss-within-envelope claim is unproven (no approved envelope exists, DEC05 open); REQ-029's restore drill ran with real numbers but is explicitly local-prototype-only</t>
+        </is>
+      </c>
       <c r="F12" s="7" t="str"/>
       <c r="G12" s="4">
         <f>IF(AND(D12="Pass",E12&lt;&gt;"",F12&lt;&gt;""),"Verified","Unverified")</f>
@@ -4395,10 +4683,14 @@
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>Not tested</t>
-        </is>
-      </c>
-      <c r="E13" s="7" t="str"/>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="E13" s="7" t="inlineStr">
+        <is>
+          <t>REQ-012's guided-authoring UI (UI08) has no frontend page yet -- fork/import/blank-creation exist only as backend endpoints</t>
+        </is>
+      </c>
       <c r="F13" s="7" t="str"/>
       <c r="G13" s="4">
         <f>IF(AND(D13="Pass",E13&lt;&gt;"",F13&lt;&gt;""),"Verified","Unverified")</f>
@@ -4424,10 +4716,14 @@
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>Not tested</t>
-        </is>
-      </c>
-      <c r="E14" s="7" t="str"/>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>REQ-010/013/014 pass; REQ-012's guided-authoring UI gap (same as AC08) keeps this from a full Pass</t>
+        </is>
+      </c>
       <c r="F14" s="7" t="str"/>
       <c r="G14" s="4">
         <f>IF(AND(D14="Pass",E14&lt;&gt;"",F14&lt;&gt;""),"Verified","Unverified")</f>
@@ -4453,10 +4749,14 @@
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>Not tested</t>
-        </is>
-      </c>
-      <c r="E15" s="7" t="str"/>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="E15" s="7" t="inlineStr">
+        <is>
+          <t>REQ-017/019/021/023 pass; REQ-024's remaining concurrency gap (exception/membership/reviewer-authority reads not locked) keeps this from a full Pass</t>
+        </is>
+      </c>
       <c r="F15" s="7" t="str"/>
       <c r="G15" s="4">
         <f>IF(AND(D15="Pass",E15&lt;&gt;"",F15&lt;&gt;""),"Verified","Unverified")</f>
@@ -4482,10 +4782,14 @@
       </c>
       <c r="D16" s="7" t="inlineStr">
         <is>
-          <t>Not tested</t>
-        </is>
-      </c>
-      <c r="E16" s="7" t="str"/>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="E16" s="7" t="inlineStr">
+        <is>
+          <t>REQ-017/018/021/022 mostly hold; REQ-020's not-applicable-vs-class-floor validation is not built at all</t>
+        </is>
+      </c>
       <c r="F16" s="7" t="str"/>
       <c r="G16" s="4">
         <f>IF(AND(D16="Pass",E16&lt;&gt;"",F16&lt;&gt;""),"Verified","Unverified")</f>
@@ -4511,10 +4815,14 @@
       </c>
       <c r="D17" s="7" t="inlineStr">
         <is>
-          <t>Not tested</t>
-        </is>
-      </c>
-      <c r="E17" s="7" t="str"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="E17" s="7" t="inlineStr">
+        <is>
+          <t>REQ-016/025 both Pass -- gate_occurrences represents each review as its own row; superseding is reason-recorded and never mutates the original</t>
+        </is>
+      </c>
       <c r="F17" s="7" t="str"/>
       <c r="G17" s="4">
         <f>IF(AND(D17="Pass",E17&lt;&gt;"",F17&lt;&gt;""),"Verified","Unverified")</f>
@@ -4540,10 +4848,14 @@
       </c>
       <c r="D18" s="7" t="inlineStr">
         <is>
-          <t>Not tested</t>
-        </is>
-      </c>
-      <c r="E18" s="7" t="str"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="E18" s="7" t="inlineStr">
+        <is>
+          <t>REQ-010/011 both Pass -- publishing a new version never edits a prior one, tested</t>
+        </is>
+      </c>
       <c r="F18" s="7" t="str"/>
       <c r="G18" s="4">
         <f>IF(AND(D18="Pass",E18&lt;&gt;"",F18&lt;&gt;""),"Verified","Unverified")</f>
@@ -4569,10 +4881,14 @@
       </c>
       <c r="D19" s="7" t="inlineStr">
         <is>
-          <t>Not tested</t>
-        </is>
-      </c>
-      <c r="E19" s="7" t="str"/>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="E19" s="7" t="inlineStr">
+        <is>
+          <t>REQ-002/003/004/005/006/031 all Pass; REQ-056 (billing tiering) is not built</t>
+        </is>
+      </c>
       <c r="F19" s="7" t="str"/>
       <c r="G19" s="4">
         <f>IF(AND(D19="Pass",E19&lt;&gt;"",F19&lt;&gt;""),"Verified","Unverified")</f>
@@ -4601,7 +4917,11 @@
           <t>Not tested</t>
         </is>
       </c>
-      <c r="E20" s="7" t="str"/>
+      <c r="E20" s="7" t="inlineStr">
+        <is>
+          <t>The tracker mechanism itself now exists and is genuinely current (this xlsx, TRACKER.md, the pm-sdlc-tracker database), but several constituent requirements (REQ-043/044/048/050/057/058) remain Not tested, so the full matrix this criterion asks for cannot yet be called complete</t>
+        </is>
+      </c>
       <c r="F20" s="7" t="str"/>
       <c r="G20" s="4">
         <f>IF(AND(D20="Pass",E20&lt;&gt;"",F20&lt;&gt;""),"Verified","Unverified")</f>
@@ -4627,10 +4947,14 @@
       </c>
       <c r="D21" s="7" t="inlineStr">
         <is>
-          <t>Not tested</t>
-        </is>
-      </c>
-      <c r="E21" s="7" t="str"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="E21" s="7" t="inlineStr">
+        <is>
+          <t>REQ-004/032 both Pass -- My work shows only authorised assignments via real role/membership checks</t>
+        </is>
+      </c>
       <c r="F21" s="7" t="str"/>
       <c r="G21" s="4">
         <f>IF(AND(D21="Pass",E21&lt;&gt;"",F21&lt;&gt;""),"Verified","Unverified")</f>
@@ -4656,10 +4980,14 @@
       </c>
       <c r="D22" s="7" t="inlineStr">
         <is>
-          <t>Not tested</t>
-        </is>
-      </c>
-      <c r="E22" s="7" t="str"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="E22" s="7" t="inlineStr">
+        <is>
+          <t>REQ-033 Pass -- guided forms with real back-navigation links, grep-confirmed</t>
+        </is>
+      </c>
       <c r="F22" s="7" t="str"/>
       <c r="G22" s="4">
         <f>IF(AND(D22="Pass",E22&lt;&gt;"",F22&lt;&gt;""),"Verified","Unverified")</f>
@@ -4685,10 +5013,14 @@
       </c>
       <c r="D23" s="7" t="inlineStr">
         <is>
-          <t>Not tested</t>
-        </is>
-      </c>
-      <c r="E23" s="7" t="str"/>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="E23" s="7" t="inlineStr">
+        <is>
+          <t>REQ-034 (save/resume) Pass; REQ-035 (pending/confirmed recovery) is Not tested -- IPA03's open finding</t>
+        </is>
+      </c>
       <c r="F23" s="7" t="str"/>
       <c r="G23" s="4">
         <f>IF(AND(D23="Pass",E23&lt;&gt;"",F23&lt;&gt;""),"Verified","Unverified")</f>
@@ -4714,10 +5046,14 @@
       </c>
       <c r="D24" s="7" t="inlineStr">
         <is>
-          <t>Not tested</t>
-        </is>
-      </c>
-      <c r="E24" s="7" t="str"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="E24" s="7" t="inlineStr">
+        <is>
+          <t>REQ-036 Pass -- blockers explain themselves in plain language with a corrective-action link</t>
+        </is>
+      </c>
       <c r="F24" s="7" t="str"/>
       <c r="G24" s="4">
         <f>IF(AND(D24="Pass",E24&lt;&gt;"",F24&lt;&gt;""),"Verified","Unverified")</f>
@@ -4743,10 +5079,14 @@
       </c>
       <c r="D25" s="7" t="inlineStr">
         <is>
-          <t>Not tested</t>
-        </is>
-      </c>
-      <c r="E25" s="7" t="str"/>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="E25" s="7" t="inlineStr">
+        <is>
+          <t>REQ-037 (permitted-progression display) Pass; REQ-042 (critical-misunderstanding blocking) not built -- Blueprint's real WP11 has not started</t>
+        </is>
+      </c>
       <c r="F25" s="7" t="str"/>
       <c r="G25" s="4">
         <f>IF(AND(D25="Pass",E25&lt;&gt;"",F25&lt;&gt;""),"Verified","Unverified")</f>
@@ -4772,10 +5112,14 @@
       </c>
       <c r="D26" s="7" t="inlineStr">
         <is>
-          <t>Not tested</t>
-        </is>
-      </c>
-      <c r="E26" s="7" t="str"/>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="E26" s="7" t="inlineStr">
+        <is>
+          <t>REQ-001/002 Pass; REQ-038's invitation-landing UI page does not exist yet (API-only)</t>
+        </is>
+      </c>
       <c r="F26" s="7" t="str"/>
       <c r="G26" s="4">
         <f>IF(AND(D26="Pass",E26&lt;&gt;"",F26&lt;&gt;""),"Verified","Unverified")</f>
@@ -4804,7 +5148,11 @@
           <t>Not tested</t>
         </is>
       </c>
-      <c r="E27" s="7" t="str"/>
+      <c r="E27" s="7" t="inlineStr">
+        <is>
+          <t>Neither REQ-040 (WCAG audit) nor REQ-041 (onboarding-time testing) has been performed -- Blueprint's real WP11 has not started</t>
+        </is>
+      </c>
       <c r="F27" s="7" t="str"/>
       <c r="G27" s="4">
         <f>IF(AND(D27="Pass",E27&lt;&gt;"",F27&lt;&gt;""),"Verified","Unverified")</f>
@@ -4833,7 +5181,11 @@
           <t>Not tested</t>
         </is>
       </c>
-      <c r="E28" s="7" t="str"/>
+      <c r="E28" s="7" t="inlineStr">
+        <is>
+          <t>REQ-039 (timezone/translation), REQ-054 (reminders) and REQ-055 (practice mode) are all Not tested/not built</t>
+        </is>
+      </c>
       <c r="F28" s="7" t="str"/>
       <c r="G28" s="4">
         <f>IF(AND(D28="Pass",E28&lt;&gt;"",F28&lt;&gt;""),"Verified","Unverified")</f>
@@ -5885,12 +6237,12 @@
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>Pass</t>
+          <t>Partial (REQ-021 holds, REQ-020 unbuilt)</t>
         </is>
       </c>
       <c r="F8" s="7" t="inlineStr">
         <is>
-          <t>WP07 exception create/revoke endpoints re-check authority/scope/expiry live on every call (app/routers/decisions.py), never trusted from a stored status field alone.</t>
+          <t>WP07 exception create/revoke endpoints re-check authority/scope/expiry live on every call (REQ-021, Pass). REQ-020's not-applicable-vs-class-floor validation is genuinely unbuilt -- grep-confirmed zero occurrences anywhere in backend/app/, corrected 2026-09-24 after the per-requirement Requirements-sheet pass caught what the earlier WP-level pass had missed.</t>
         </is>
       </c>
       <c r="G8" s="7" t="str"/>

</xml_diff>

<commit_message>
Transcribe kenAddme's DEC05/06/07/08/11/12 answers, accepted by delivery lead
Companion doc BGP_DEC_Resolution_Intake_2026-09-25_ANSWERED.md holds the
full answer content; the approved xlsx Decisions sheet moves those six rows
to Decided with it. Same DEC01/DEC04 pattern: the delivery lead accepting
content in conversation is not an independent role sign-off and not a
tracker_cli.py gate decision. Two open items from the answer document are
carried forward, not smoothed over -- DEC05's Candidate A+ is a synthesis
needing explicit confirmation at review, and DEC11 Q19's break-glass
tenant-visibility default is flagged by the document itself as not settled.

IPA02/IPA04 in docs/DEFECT_REGISTER.md stay Open -- content answers aren't
built UI or performed assurance/durability work.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/blueprint/Build_Governance_Platform_Implementation_Tracker_v0.2_Approved.xlsx
+++ b/docs/blueprint/Build_Governance_Platform_Implementation_Tracker_v0.2_Approved.xlsx
@@ -6689,26 +6689,26 @@
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>Approved zero-loss objective within an explicit failure envelope and independent integrity verification. Candidate A versus B, covered failures and custody remain to be selected.</t>
+          <t>Decided 2026-09-27 (kenAddme's supplied answer, accepted by the delivery lead -- not an independent Operations/security-leads sign-off): Candidate A+ -- neither original candidate as framed, a synthesis of synchronous durable replication before acknowledgement (clean, truthful 'Recorded' response) plus an asynchronous independently-protected hash-chain anchor for tamper-evidence; Candidate B's pending-and-reconcile pattern survives only as a labelled, alerting degraded fallback when the sync replica is unavailable, never counted as a recorded decision. Failure scenarios covered: process crash, node failure, storage failure, single-zone failure (zero acknowledged-decision loss); regional failure via continuous archiving to a second region (RPO&lt;=5min, restored inside RTO). Explicitly NOT covered by durability alone: logical corruption from a code defect or an authorised-but-malicious write (detected by the hash chain, recovered by point-in-time restore, not prevented by replication), and simultaneous loss of the primary region and its archive. Integrity-verification mechanism is independent: the chain anchor writes to object-lock (WORM) storage under a credential the application database role cannot overwrite/delete; verification runs under a third, separate identity. Numeric targets: availability 99.5% monthly; RPO 0 in-region, &lt;=5min cross-region; RTO 8 hours; quarterly restore test into a clean environment; integrity verification at least daily, a chain mismatch treated as an S1 incident acknowledged within 1 hour. Acknowledgement is synchronous: the API returns success only once the decision row, audit entry and chain link are committed in one transaction and confirmed on a same-region different-zone synchronous replica. FLAGGED, NOT SETTLED BY THIS ANSWER ALONE: Candidate A+ is a synthesis not offered as an option in the original intake framing -- Operations/security leads still need to confirm what they are actually being asked to approve, since it isn't literally 'A or B.'</t>
         </is>
       </c>
       <c r="F10" s="7" t="inlineStr">
         <is>
-          <t>Partly decided</t>
+          <t>Decided</t>
         </is>
       </c>
       <c r="G10" s="7" t="inlineStr">
         <is>
-          <t>Named owner assigned 2026-09-25: kenAddme (active GitHub collaborator, real APPROVED reviews on PR#5/#6/#7, checked via gh pr view). Responsible for driving this decision to actual resolution -- this is an OWNERSHIP ASSIGNMENT ONLY, not the decision itself: Candidate A vs. Candidate B, covered failure scenarios, and custody for DEC05's durability mechanism remains unspecified until kenAddme (or whoever actually holds the role: Operations and security leads) supplies it. Status/Decision record/Approval date deliberately left untouched -- do not read this cell as the decision having been made.</t>
+          <t>Named owner assigned 2026-09-25: kenAddme (active GitHub collaborator, real APPROVED reviews on PR#5/#6/#7, checked via gh pr view). Responsible for driving this decision to actual resolution -- this is an OWNERSHIP ASSIGNMENT ONLY, not the decision itself: Candidate A vs. Candidate B, covered failure scenarios, and custody for DEC05's durability mechanism remains unspecified until kenAddme (or whoever actually holds the role: Operations and security leads) supplies it. Status/Decision record/Approval date deliberately left untouched -- do not read this cell as the decision having been made. kenAddme's substantive answer received 2026-09-25/27 (docs/blueprint/BGP_DEC_Resolution_Intake_2026-09-25_ANSWERED.md) and accepted by the delivery lead in conversation 2026-09-27 -- still not an independent Operations/security-leads sign-off. The answer document itself flags the Candidate A+ framing as needing explicit confirmation at review -- see 'Open items' in the answered doc.</t>
         </is>
       </c>
       <c r="H10" s="7" t="inlineStr">
         <is>
-          <t>APR-001; Blueprint v0.2 Sections 7 and 9; user approval in conversation</t>
+          <t>APR-001; Blueprint v0.2 Sections 7 and 9; user approval in conversation; docs/blueprint/BGP_DEC_Resolution_Intake_2026-09-25_ANSWERED.md (accepted 2026-09-27)</t>
         </is>
       </c>
       <c r="I10" s="12" t="n">
-        <v>46280</v>
+        <v>46292</v>
       </c>
     </row>
     <row r="11" ht="115" customHeight="1">
@@ -6734,26 +6734,26 @@
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>Approved retention review, attribution and disposal controls. Retention periods and the permanent-record conflict remain to be resolved before implementation.</t>
+          <t>Decided 2026-09-27 (kenAddme's supplied answer, accepted by the delivery lead -- not an independent Privacy-reviewer/owner sign-off): retention periods differ by record type as a floor tenants may lengthen but not shorten -- decisions/gate approvals/exceptions 7yrs after Gate 6; requirements/designs/acceptance/release records life-of-service+3yrs (never &lt;7yrs after Gate 6); audit events 7yrs after Gate 6 or after the event, whichever is later; attachment bytes shortest of all, default 3yrs, tenant-configurable, purgeable early while metadata/hash survive. REQ-025's permanent-record guarantee narrowed to structural fields only (actor id, timestamp, action, before/after hashes in decisions/gate_decisions/audit_events -- never mutable); redaction permitted only on named personal-data fields and attachment bytes, implemented as a chain-re-anchored redaction event (proves a redaction happened without revealing what was redacted) -- one narrow, genuine exception, not a blanket one. Actor stored as a stable pseudonymous id with the id-to-person mapping in one separately-redactable table so an erasure request doesn't break a chain. True end-of-retention disposal removes the row set and leaves a tombstone (record id, hash, disposal date, authoriser, method). Legal hold: placed by the tenant's named records custodian/data owner or the project sponsor (platform operator only on written legal instruction, tenant notified it exists); overrides all scheduled disposal/shortening/purge but not a legally compelled erasure request (routed to legal advice instead). Mandatory hold fields: scope/reason/owner/placed date/release condition; release needs the same role and its own record. Other specifics: deleted users keep attribution via stable id + display-name snapshot; exports pseudonymous by default; disposal effective in live data within 24h, in backups within the backup retention window (no false instant-deletion claim).</t>
         </is>
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>Partly decided</t>
+          <t>Decided</t>
         </is>
       </c>
       <c r="G11" s="7" t="inlineStr">
         <is>
-          <t>Named owner assigned 2026-09-25: kenAddme (active GitHub collaborator, real APPROVED reviews on PR#5/#6/#7, checked via gh pr view). Responsible for driving this decision to actual resolution -- this is an OWNERSHIP ASSIGNMENT ONLY, not the decision itself: actual retention periods and the permanent-record conflict for DEC06 remains unspecified until kenAddme (or whoever actually holds the role: Privacy reviewer and owner) supplies it. Status/Decision record/Approval date deliberately left untouched -- do not read this cell as the decision having been made.</t>
+          <t>Named owner assigned 2026-09-25: kenAddme (active GitHub collaborator, real APPROVED reviews on PR#5/#6/#7, checked via gh pr view). Responsible for driving this decision to actual resolution -- this is an OWNERSHIP ASSIGNMENT ONLY, not the decision itself: actual retention periods and the permanent-record conflict for DEC06 remains unspecified until kenAddme (or whoever actually holds the role: Privacy reviewer and owner) supplies it. Status/Decision record/Approval date deliberately left untouched -- do not read this cell as the decision having been made. kenAddme's substantive answer received 2026-09-25/27 (docs/blueprint/BGP_DEC_Resolution_Intake_2026-09-25_ANSWERED.md) and accepted by the delivery lead in conversation 2026-09-27 -- still not an independent Privacy-reviewer/owner sign-off.</t>
         </is>
       </c>
       <c r="H11" s="7" t="inlineStr">
         <is>
-          <t>APR-001; Blueprint v0.2 Sections 7 and 9; user approval in conversation</t>
+          <t>APR-001; Blueprint v0.2 Sections 7 and 9; user approval in conversation; docs/blueprint/BGP_DEC_Resolution_Intake_2026-09-25_ANSWERED.md (accepted 2026-09-27)</t>
         </is>
       </c>
       <c r="I11" s="12" t="n">
-        <v>46280</v>
+        <v>46292</v>
       </c>
     </row>
     <row r="12" ht="115" customHeight="1">
@@ -6779,26 +6779,26 @@
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>Approved declarative rule schema and evaluation order in Section 5.5. Vocabulary limits, third framework and its permitted use remain to be specified.</t>
+          <t>Decided 2026-09-27 (kenAddme's supplied answer, accepted by the delivery lead -- not an independent Technical-lead sign-off): current vocabulary (eq/in/all/any, depth 5, no eval/exec) approved as-is, plus additions -- not (negation), gte/lte (dates/counts), count(...) with a comparison ('at least N of these complete') -- and two tightenings: cap total condition nodes at 200 in addition to depth-5, and a hard evaluation timeout; rules are pure functions of project state plus a supplied 'as at' timestamp (no external calls, no wall-clock reads inside a rule). vocabulary_version stamped on every template version so old templates evaluate identically forever. Third permitted framework fixture: an agile Definition-of-Ready/Definition-of-Done framework with no gates at all (recurring per-increment checks, unnumbered, evaluated every sprint) -- deliberately the harder, structurally-different test; second choice if an external standard is preferred: NIST SSDF 800-218 practice groups. Scope: full parity with the other two fixtures (tracks/items/rules/roles/statuses/decisions) -- marked a validation fixture, not a shipped starter template, until it passes its own review.</t>
         </is>
       </c>
       <c r="F12" s="7" t="inlineStr">
         <is>
-          <t>Partly decided</t>
+          <t>Decided</t>
         </is>
       </c>
       <c r="G12" s="7" t="inlineStr">
         <is>
-          <t>Named owner assigned 2026-09-25: kenAddme (active GitHub collaborator, real APPROVED reviews on PR#5/#6/#7, checked via gh pr view). Responsible for driving this decision to actual resolution -- this is an OWNERSHIP ASSIGNMENT ONLY, not the decision itself: vocabulary limits and the third permitted framework for DEC07 remains unspecified until kenAddme (or whoever actually holds the role: Technical lead) supplies it. Status/Decision record/Approval date deliberately left untouched -- do not read this cell as the decision having been made.</t>
+          <t>Named owner assigned 2026-09-25: kenAddme (active GitHub collaborator, real APPROVED reviews on PR#5/#6/#7, checked via gh pr view). Responsible for driving this decision to actual resolution -- this is an OWNERSHIP ASSIGNMENT ONLY, not the decision itself: vocabulary limits and the third permitted framework for DEC07 remains unspecified until kenAddme (or whoever actually holds the role: Technical lead) supplies it. Status/Decision record/Approval date deliberately left untouched -- do not read this cell as the decision having been made. kenAddme's substantive answer received 2026-09-25/27 (docs/blueprint/BGP_DEC_Resolution_Intake_2026-09-25_ANSWERED.md) and accepted by the delivery lead in conversation 2026-09-27 -- still not an independent Technical-lead sign-off.</t>
         </is>
       </c>
       <c r="H12" s="7" t="inlineStr">
         <is>
-          <t>APR-001; Blueprint v0.2 Sections 7 and 9; user approval in conversation</t>
+          <t>APR-001; Blueprint v0.2 Sections 7 and 9; user approval in conversation; docs/blueprint/BGP_DEC_Resolution_Intake_2026-09-25_ANSWERED.md (accepted 2026-09-27)</t>
         </is>
       </c>
       <c r="I12" s="12" t="n">
-        <v>46280</v>
+        <v>46292</v>
       </c>
     </row>
     <row r="13" ht="115" customHeight="1">
@@ -6824,26 +6824,26 @@
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>Approved 90% unaided task completion separately for each user group and twenty-minute onboarding. Sample sizes, devices, network profile and numeric performance budgets remain to be specified.</t>
+          <t>Decided 2026-09-27 (kenAddme's supplied answer, accepted by the delivery lead -- not an independent UX/technical-leads sign-off): sample sizes -- beginner 8, contributor 5, client approver 5, administrator 5 (23 total); disabled/assistive-technology users distributed across the four groups (&gt;=5 total) plus a dedicated expert accessibility review, not a separate fifth group; &gt;=6 participants on older/low-end devices, similarly distributed. Device/network profiles: primary budget target mid-range Android on Fast 3G (1.6Mbps/150ms RTT, the realistic Ghanaian mobile case); degraded acceptance case low-end Android (~4GB RAM, 2019-era) on Slow 3G (400kbps/400ms RTT), which must stay usable not fast; also an iPhone 2-3 generations old on 4G, desktop broadband baseline, 320px/360px viewports, 400% zoom reflow (WCAG 1.4.10). API p95 latency budgets (server time at origin): reads (gate view/dashboard) p95&lt;=300ms/p99&lt;=800ms; ordinary writes p95&lt;=500ms; decision writes p95&lt;=800ms/p99&lt;=1.5s (the allowance DEC05's synchronous replica commit needs); exports asynchronous, must begin streaming within 2s. Page/render budget: critical render path &lt;=170KB compressed; total first load &lt;=350KB, heaviest authoring screen &lt;=1MB; LCP&lt;=2.5s primary/&lt;=5s degraded; INP&lt;=200ms; CLS&lt;=0.1; no more than two blocking requests before first render -- all enforced in CI as a blocking budget check, not a dashboard someone reads occasionally.</t>
         </is>
       </c>
       <c r="F13" s="7" t="inlineStr">
         <is>
-          <t>Partly decided</t>
+          <t>Decided</t>
         </is>
       </c>
       <c r="G13" s="7" t="inlineStr">
         <is>
-          <t>Named owner assigned 2026-09-25: kenAddme (active GitHub collaborator, real APPROVED reviews on PR#5/#6/#7, checked via gh pr view). Responsible for driving this decision to actual resolution -- this is an OWNERSHIP ASSIGNMENT ONLY, not the decision itself: sample sizes, device/network profiles and numeric performance budgets for DEC08 remains unspecified until kenAddme (or whoever actually holds the role: UX and technical leads) supplies it. Status/Decision record/Approval date deliberately left untouched -- do not read this cell as the decision having been made.</t>
+          <t>Named owner assigned 2026-09-25: kenAddme (active GitHub collaborator, real APPROVED reviews on PR#5/#6/#7, checked via gh pr view). Responsible for driving this decision to actual resolution -- this is an OWNERSHIP ASSIGNMENT ONLY, not the decision itself: sample sizes, device/network profiles and numeric performance budgets for DEC08 remains unspecified until kenAddme (or whoever actually holds the role: UX and technical leads) supplies it. Status/Decision record/Approval date deliberately left untouched -- do not read this cell as the decision having been made. kenAddme's substantive answer received 2026-09-25/27 (docs/blueprint/BGP_DEC_Resolution_Intake_2026-09-25_ANSWERED.md) and accepted by the delivery lead in conversation 2026-09-27 -- still not an independent UX/technical-leads sign-off.</t>
         </is>
       </c>
       <c r="H13" s="7" t="inlineStr">
         <is>
-          <t>APR-001; Blueprint v0.2 Sections 7 and 9; user approval in conversation</t>
+          <t>APR-001; Blueprint v0.2 Sections 7 and 9; user approval in conversation; docs/blueprint/BGP_DEC_Resolution_Intake_2026-09-25_ANSWERED.md (accepted 2026-09-27)</t>
         </is>
       </c>
       <c r="I13" s="12" t="n">
-        <v>46280</v>
+        <v>46292</v>
       </c>
     </row>
     <row r="14" ht="115" customHeight="1">
@@ -6951,26 +6951,26 @@
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>Approved no routine operator evidence access and no decision-edit authority. Break-glass scope, approval path, tenant visibility and independent key custody remain to be specified.</t>
+          <t>Decided 2026-09-27 (kenAddme's supplied answer, accepted by the delivery lead -- not an independent Security-lead/owner sign-off): routine operator access is tenant metadata, aggregate health, and error traces with tenant content redacted -- never evidence, attachments, decision content or personal data. Break-glass adds, time-boxed to one incident: read specific rows for one named incident; read one attachment only where the incident concerns that specific attachment; run a scoped data-fix migration -- never editing/deleting a decision, disabling audit, exporting a whole tenant, or touching more than one tenant in a session; sessions expire in 60 minutes, bound to one tenant and one incident id, every query logged. Approval: two-person rule (requester + an approver who is not the requester, holding Security Lead or Executive/Service Owner; out of hours, named Service Owner primary / Technical Lead or on-call deputy); incident id mandatory; approval recorded before access, or (if the granting system itself is down) a recorded verbal approval with written confirmation inside 24 hours; retrospective review within 72 hours. OPEN ITEM, EXPLICITLY NOT SETTLED BY THIS ANSWER ALONE (the answer document's own words): tenant-visibility default for break-glass is recommended as tenant pre-approval by default, with a narrow life-safety/legal-compulsion carve-out (immediate access, tenant notified when the session opens) -- but this is presented as 'Security lead/owner's call to make, not a settled fact,' a genuine privacy-vs-incident-response-speed trade-off. Either way: the session appears in the tenant's own audit log (who/when/incident/scope/what was read/approver/close time), a report follows within 72 hours, no suppression window, no silent access. Key custody: three separate identities against a managed KMS/HSM -- application role (request decrypt only), key custodian (rotate/create keys, no data read), operator role (neither power). Custodian is a named person distinct from on-call with a named deputy; backup-encryption keys and the chain-anchor write credential live in a separate account from production under object-lock (even the custodian can't delete anchors inside their retention period); key deletion/rotation needs the same two-person approval as break-glass, reviewed as part of the quarterly access review.</t>
         </is>
       </c>
       <c r="F16" s="7" t="inlineStr">
         <is>
-          <t>Partly decided</t>
+          <t>Decided</t>
         </is>
       </c>
       <c r="G16" s="7" t="inlineStr">
         <is>
-          <t>Named owner assigned 2026-09-25: kenAddme (active GitHub collaborator, real APPROVED reviews on PR#5/#6/#7, checked via gh pr view). Responsible for driving this decision to actual resolution -- this is an OWNERSHIP ASSIGNMENT ONLY, not the decision itself: break-glass scope, approval path, tenant visibility and independent key custody for DEC11 remains unspecified until kenAddme (or whoever actually holds the role: Security lead and owner) supplies it. Status/Decision record/Approval date deliberately left untouched -- do not read this cell as the decision having been made.</t>
+          <t>Named owner assigned 2026-09-25: kenAddme (active GitHub collaborator, real APPROVED reviews on PR#5/#6/#7, checked via gh pr view). Responsible for driving this decision to actual resolution -- this is an OWNERSHIP ASSIGNMENT ONLY, not the decision itself: break-glass scope, approval path, tenant visibility and independent key custody for DEC11 remains unspecified until kenAddme (or whoever actually holds the role: Security lead and owner) supplies it. Status/Decision record/Approval date deliberately left untouched -- do not read this cell as the decision having been made. kenAddme's substantive answer received 2026-09-25/27 (docs/blueprint/BGP_DEC_Resolution_Intake_2026-09-25_ANSWERED.md) and accepted by the delivery lead in conversation 2026-09-27 -- still not an independent Security-lead/owner sign-off. The answer document itself flags DEC11 Q19's break-glass tenant-visibility default as 'Security lead/owner's call to make, not a settled fact' -- see 'Open items' in the answered doc.</t>
         </is>
       </c>
       <c r="H16" s="7" t="inlineStr">
         <is>
-          <t>APR-001; Blueprint v0.2 Sections 7 and 9; user approval in conversation</t>
+          <t>APR-001; Blueprint v0.2 Sections 7 and 9; user approval in conversation; docs/blueprint/BGP_DEC_Resolution_Intake_2026-09-25_ANSWERED.md (accepted 2026-09-27)</t>
         </is>
       </c>
       <c r="I16" s="12" t="n">
-        <v>46280</v>
+        <v>46292</v>
       </c>
     </row>
     <row r="17" ht="115" customHeight="1">
@@ -6996,7 +6996,7 @@
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>Approved provenance-preserving migration policy; never invent missing actors or approvals. Any real-data import still requires data-owner authorisation and reconciliation evidence.</t>
+          <t>Approved provenance-preserving migration policy; never invent missing actors or approvals. Any real-data import still requires data-owner authorisation and reconciliation evidence. REFINED 2026-09-27 (kenAddme's supplied answer, accepted by the delivery lead): KenAddme IT Links is data owner/controller for records it created for its own purposes (Freston Kenny Adedeme as named custodian) -- but where a legacy record holds client personal data processed on the client's instruction, the CLIENT is controller and KenAddme is processor for that record; classify each import per record set, not wholesale, and carve out client-owned records needing client authorisation before import. Platform-side mirror: on the platform itself the tenant is controller and the operator is processor, so KenAddme-as-tenant is data owner of its own tenant data while KenAddme-as-operator is not. Substantive authorisation/reconciliation evidence for any real import -- BEFORE: written import authorisation naming source system/record set/lawful basis/destination tenant/data classification/client consents, a source data inventory, a privacy screen confirming no Restricted data (or documented approval if there is), a dry run into non-production with the reconciliation report reviewed. DURING: a dedicated time-limited migration identity (not operator/application role), every write tagged with a batch id. AFTER: counts source-vs-destination by type with a zero-variance statement or explained variance list, a hash comparison of normalised source rows, manual field-by-field verification of the greater of 10% or 30 records by someone other than the importer, a new chain checkpoint covering the imported set, the source frozen read-only at cut-over. The requirement that matters most: every imported decision must carry its original actor and timestamp, or be imported as 'attributed: unknown, migrated' -- never assigned to whoever ran the import; every imported row flagged 'origin: migrated' permanently. Sign-off: data owner plus an independent reviewer, recorded as a change record, not a routine operation.</t>
         </is>
       </c>
       <c r="F17" s="7" t="inlineStr">
@@ -7006,16 +7006,16 @@
       </c>
       <c r="G17" s="7" t="inlineStr">
         <is>
-          <t>Named owner assigned 2026-09-25: kenAddme (active GitHub collaborator, real APPROVED reviews on PR#5/#6/#7, checked via gh pr view). Responsible for driving this decision to actual resolution -- this is an OWNERSHIP ASSIGNMENT ONLY, not the decision itself: the named Data owner who will actually authorise and reconcile each real import under DEC12's already-decided policy remains unspecified until kenAddme (or whoever actually holds the role: Data owner) supplies it. Status/Decision record/Approval date deliberately left untouched -- do not read this cell as the decision having been made.</t>
+          <t>Named owner assigned 2026-09-25: kenAddme (active GitHub collaborator, real APPROVED reviews on PR#5/#6/#7, checked via gh pr view). Responsible for driving this decision to actual resolution -- this is an OWNERSHIP ASSIGNMENT ONLY, not the decision itself: the named Data owner who will actually authorise and reconcile each real import under DEC12's already-decided policy remains unspecified until kenAddme (or whoever actually holds the role: Data owner) supplies it. Status/Decision record/Approval date deliberately left untouched -- do not read this cell as the decision having been made. kenAddme's substantive answer received 2026-09-25/27 (docs/blueprint/BGP_DEC_Resolution_Intake_2026-09-25_ANSWERED.md) and accepted by the delivery lead in conversation 2026-09-27 -- still not an independent Data-owner sign-off.</t>
         </is>
       </c>
       <c r="H17" s="7" t="inlineStr">
         <is>
-          <t>APR-001; Blueprint v0.2 Sections 7 and 9; user approval in conversation</t>
+          <t>APR-001; Blueprint v0.2 Sections 7 and 9; user approval in conversation; docs/blueprint/BGP_DEC_Resolution_Intake_2026-09-25_ANSWERED.md (accepted 2026-09-27)</t>
         </is>
       </c>
       <c r="I17" s="12" t="n">
-        <v>46280</v>
+        <v>46292</v>
       </c>
     </row>
   </sheetData>

</xml_diff>